<commit_message>
Publish q2792 Airflow Windows WSL2 reproduction
</commit_message>
<xml_diff>
--- a/task/任务规格转化.xlsx
+++ b/task/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R56d757d26df041be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="Reb5177aa00354341"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -383,41 +383,49 @@
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="5" t="str">
-        <x:v>Airflow对象读取</x:v>
+        <x:v>窗口交接</x:v>
       </x:c>
       <x:c r="B14" s="5" t="str">
-        <x:v>dag_inventory.csv从DagBag的DAG和任务对象生成，dependency_inventory.csv从ExternalTaskSensor实例生成</x:v>
+        <x:v>release_handoff.csv记录变更窗口、影响范围、等待预算、启用方式、回滚条件和观察指标</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="5" t="str">
-        <x:v>岗位消费</x:v>
+        <x:v>Airflow对象读取</x:v>
       </x:c>
       <x:c r="B15" s="5" t="str">
-        <x:v>版本负责人接收DAG源码和结构清单，维护窗值班使用发布顺序并负责现场启用、补跑与历史清理</x:v>
+        <x:v>dag_inventory.csv从DagBag的DAG和任务对象生成，dependency_inventory.csv从ExternalTaskSensor实例生成</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="5" t="str">
-        <x:v>完成条件</x:v>
+        <x:v>岗位消费</x:v>
       </x:c>
       <x:c r="B16" s="5" t="str">
-        <x:v>三条DAG可由DagBag导入，任务图与输入身份闭合，Sensor属性和逻辑日期与计划一致</x:v>
+        <x:v>版本负责人接收DAG源码和清单，维护窗值班负责启用、指标观察和条件回滚，补跑与历史清理另行处理</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="5" t="str">
+        <x:v>完成条件</x:v>
+      </x:c>
+      <x:c r="B17" s="5" t="str">
+        <x:v>三条DAG可由DagBag导入，任务图与输入身份闭合，Sensor属性、逻辑日期和窗口交接与申请一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="5" t="str">
         <x:v>可验证点</x:v>
       </x:c>
-      <x:c r="B17" s="5" t="str">
-        <x:v>DAG身份、任务边、日程属性、Sensor目标、状态集合、等待属性、逻辑日期和三份清单之间的业务键</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="15" hidden="0" customHeight="1">
-      <x:c r="A18" s="6" t="str">
+      <x:c r="B18" s="5" t="str">
+        <x:v>DAG身份、任务边、日程属性、Sensor目标、状态集合、等待属性、逻辑日期、发布字段和四份清单之间的业务键</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="6" t="str">
         <x:v>不适合作为评分点的内容</x:v>
       </x:c>
-      <x:c r="B18" s="6" t="str">
+      <x:c r="B19" s="6" t="str">
         <x:v>源码排版、变量命名、导入顺序、CSV行序、编辑器和临时AIRFLOW_HOME路径</x:v>
       </x:c>
     </x:row>

</xml_diff>